<commit_message>
Haberleşme grubuna "Mayday Main Module" eklendi.
</commit_message>
<xml_diff>
--- a/pages/haberlesme.xlsx
+++ b/pages/haberlesme.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MTK\Butkon\Projeler\BTK42_EXCEL\pages\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Depom\Projects\_GithubIO\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FF6446-DAF5-407D-BC2D-0EBDB5730769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D628C0-0E51-4B61-AC8D-81DEC906D0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="46">
   <si>
     <t>Sıra</t>
   </si>
@@ -154,6 +154,15 @@
   </si>
   <si>
     <t>https://github.com/btk42/CM-MLI-00-000-000-P1B1-01</t>
+  </si>
+  <si>
+    <t>CM-MDY-00-000-MCR-H3B0-01</t>
+  </si>
+  <si>
+    <t>Mayday</t>
+  </si>
+  <si>
+    <t>https://github.com/btk42/CM-MDY-00-000-MCR-H3B0-01</t>
   </si>
 </sst>
 </file>
@@ -540,7 +549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="6" bestFit="1" customWidth="1"/>
@@ -924,12 +933,100 @@
       </c>
       <c r="K11" s="5"/>
     </row>
+    <row r="12" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+    </row>
+    <row r="14" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+    </row>
+    <row r="15" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+    </row>
+    <row r="16" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="K9" r:id="rId1" xr:uid="{473CCB9F-9F6A-4388-BAD8-F0D74455EE1C}"/>
+    <hyperlink ref="K12" r:id="rId2" xr:uid="{3BBB5629-1937-4FDF-9F32-CCFC157F4AD6}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Sayfa &amp;P</oddFooter>

</xml_diff>